<commit_message>
finish tc module Home
</commit_message>
<xml_diff>
--- a/Doc_app/Test_case_ME_IOS.xlsx
+++ b/Doc_app/Test_case_ME_IOS.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="121">
   <si>
     <t>ID</t>
   </si>
@@ -93,57 +93,62 @@
 - Không bị vỡ layout trong trường hợp lage-text mode (accessibility setting) được bật</t>
   </si>
   <si>
-    <t>F_H_01</t>
-  </si>
-  <si>
-    <t>Kiểm tra khả năng điều hướng từ màn Home sang các module khác</t>
+    <t>kiểm thử điều hướng - ID chung: F_H_01</t>
+  </si>
+  <si>
+    <t>F_H_SET</t>
+  </si>
+  <si>
+    <t>Kiểm tra khả năng điều hướng từ màn Home sang module "App Setting"</t>
   </si>
   <si>
     <t>- màn "Home"
 - đã cấp quyền đầy đủ</t>
   </si>
   <si>
-    <t>1.a. chọn button "Setting"</t>
+    <t>1. chọn button "Setting"</t>
   </si>
   <si>
     <t>- chuyển sang màn "Setting"</t>
   </si>
   <si>
-    <t>sub-ID: F_H_SET</t>
-  </si>
-  <si>
-    <t>1.b. điều hướng sang module "Remove objects"bằng 1 trong các cách sau:
-1.b.1. chọn image carousel khi hiện baner "Remove Object"
-1.b.2. chọn button "Remove object" ở fearture compact view
-1.b.3. chọn banner "Remove object" ở topic "AI Tool"
-1.b.4. chọn button "Remove object" ở mục "Rencently Used"(nếu có)</t>
+    <t>F_H_RO</t>
+  </si>
+  <si>
+    <t>Kiểm tra khả năng điều hướng từ màn Home sang module "Remove Object"</t>
+  </si>
+  <si>
+    <t>1. điều hướng sang module "Remove objects"bằng 1 trong các cách sau:
+1.a. chọn image carousel khi hiện baner "Remove Object"
+1.b. chọn button "Remove object" ở fearture compact view
+1.c. chọn banner "Remove object" ở topic "AI Tool"
+1.d. chọn button "Remove object" ở mục "Rencently Used"(nếu có)</t>
   </si>
   <si>
     <t>- hiện dialog "Choose Image"</t>
   </si>
   <si>
-    <t>sub-ID: F_H_RO</t>
-  </si>
-  <si>
-    <t>2.b. chọn 1 ảnh bất kỳ</t>
+    <t>2. chọn 1 ảnh bất kỳ</t>
   </si>
   <si>
     <t>- chuyển sang màn "Remove Objects"
 - ảnh input load thành công, đúng orientation, không xoay sai chiều</t>
   </si>
   <si>
-    <t>1.c. điều hướng sang module "Edit Background"/"Remove Background" bằng 1 trong các cách sau:
-1.c.1. chọn image carousel khi hiện baner "Edit Background"
-1.c.2. chọn button "Edit Background" ở fearture compact view
-1.c.3. chọn banner "Edit Background" ở topic "AI Tool"
-1.c.4. chọn button "Edit Background" ở mục "Recently Used" (nếu có)</t>
-  </si>
-  <si>
-    <t>sub-ID: F_H_RB_01
-- điều hướng:  "Home" -&gt; "Background" Home</t>
-  </si>
-  <si>
-    <t>2.c. chọn 1 ảnh bất kỳ</t>
+    <t>F_H_RB_01</t>
+  </si>
+  <si>
+    <t>Kiểm tra khả năng điều hướng từ màn Home sang module "Edit  Background"</t>
+  </si>
+  <si>
+    <t>1. điều hướng sang module "Edit Background"/"Remove Background" bằng 1 trong các cách sau:
+1.a. chọn image carousel khi hiện baner "Edit Background"
+1.b. chọn button "Edit Background" ở fearture compact view
+1.c. chọn banner "Edit Background" ở topic "AI Tool"
+1.d. chọn button "Edit Background" ở mục "Recently Used" (nếu có)</t>
+  </si>
+  <si>
+    <t>- screen:  "Home" -&gt; "Background" Home</t>
   </si>
   <si>
     <t>- hiện dialog "Processing" -&gt; chuyển sang màn "Background Home"
@@ -161,17 +166,16 @@
     <t>- không có kết nối internet</t>
   </si>
   <si>
-    <t>1.d. chọn 1 template bất kỳ ở topic "Background"</t>
+    <t>F_H_RB_02</t>
+  </si>
+  <si>
+    <t>1. chọn 1 template bất kỳ ở topic "Background"</t>
   </si>
   <si>
     <t>- hiện dialog "Choose image"</t>
   </si>
   <si>
-    <t>sub-ID: F_H_RB_02 
-- điều hướng: "Home" -&gt; "Background Editor"</t>
-  </si>
-  <si>
-    <t>2.d. chọn 1 ảnh bất kỳ</t>
+    <t>- điều hướng: "Home" -&gt; "Background Editor"</t>
   </si>
   <si>
     <t>- hiện dialog "Processing" -&gt; chuyển sang màn "Background Editor"
@@ -179,7 +183,10 @@
 - load thành công, đúng template đã chọn</t>
   </si>
   <si>
-    <t>1.e. chọn 1 tempalate bất kỳ ở topic "Design"</t>
+    <t>F_H_RB_03</t>
+  </si>
+  <si>
+    <t>1. chọn 1 tempalate bất kỳ ở topic "Design"</t>
   </si>
   <si>
     <t>- sang màn "Background Editor"
@@ -187,14 +194,10 @@
 - frontground có button "replace"</t>
   </si>
   <si>
-    <t>sub-ID: F_H_RB_03 
-- điều hướng: "Home" -&gt; "Background Editor"</t>
-  </si>
-  <si>
-    <t>2.e. chọn button "replace"</t>
-  </si>
-  <si>
-    <t>3.e chọn 1 ảnh bất kỳ</t>
+    <t>2. chọn button "replace"</t>
+  </si>
+  <si>
+    <t>3. chọn 1 ảnh bất kỳ</t>
   </si>
   <si>
     <t>- hiện dialog"Processing" -&gt; quay về màn "Background Editor"
@@ -204,17 +207,17 @@
     <t>- hiện modal "Error": check your internet</t>
   </si>
   <si>
-    <t>1.f. điều hướng sang module "Basic Edit" bằng 1 trong các cách sau đây:
-1.f.1. chọn button "Start Editing" trên fearture compact view
-1.f.2. chọn button "Basic Edit" trên fearture compact view
-1.f.3. chọn banner "Basic Edit" ở mục "AI Tools"
-1.f.4. chọn button "Basic Edit" ở mục "Recently used"</t>
-  </si>
-  <si>
-    <t>Sub-ID: F_H_BE_01</t>
-  </si>
-  <si>
-    <t>2.f. chọn 1 ảnh bất kỳ</t>
+    <t>F_H_BE_01</t>
+  </si>
+  <si>
+    <t>Kiểm tra khả năng điều hướng từ màn Home sang module "Basic Edit"</t>
+  </si>
+  <si>
+    <t>1. điều hướng sang module "Basic Edit" bằng 1 trong các cách sau đây:
+1.a. chọn button "Start Editing" trên fearture compact view
+1.b. chọn button "Basic Edit" trên fearture compact view
+1.c. chọn banner "Basic Edit" ở mục "AI Tools"
+1.d. chọn button "Basic Edit" ở mục "Recently used"</t>
   </si>
   <si>
     <t>- sang màn "Basic Edit"
@@ -223,14 +226,11 @@
 - non-pro acount: các tool button "AI Fill", "AI Expand" được đính badge "Pro"</t>
   </si>
   <si>
-    <t>1.g. điều hướng sang module "Basic Edit" với các tool đã được bật sẵn bằng cách chọn các button sau: 
+    <t>F_H_BE_02</t>
+  </si>
+  <si>
+    <t>1. điều hướng sang module "Basic Edit" với các tool đã được bật sẵn bằng cách chọn các button sau: 
 "Frame", "Filter", "Adjust", "Blur", "Texture", "Brushes", "Crop", "Text", "Sticker"</t>
-  </si>
-  <si>
-    <t>sub-ID: F_H_BE_02</t>
-  </si>
-  <si>
-    <t>2.g. chọn 1 ảnh bất kỳ</t>
   </si>
   <si>
     <t>- sang màn "Basic Edit"
@@ -238,17 +238,17 @@
 - tool bottom sheet tương ứng với fearture đã chọn (ở step 1) hiện trên màn hình với 1 option default đã được chọn</t>
   </si>
   <si>
-    <t>1.h. điều hướng sang module "AI Enhance" bằng 1 trong các cách sau: 
-1.h.1. chọn image carousel khi hiện banner "AI Enhance"
-1.h.2. chọn button "AI Enhance" ở fearture compact view 
-1.h.3. chọn banner "AI Enhance" ở mục "AI Tools"
-1.h.4. chọn button "AI Enhance" ở mục "Recently Used" (nếu có)</t>
-  </si>
-  <si>
-    <t>sub-ID: F_H_AE</t>
-  </si>
-  <si>
-    <t>2.h. chọn 1 ảnh bất kỳ</t>
+    <t>F_H_AE</t>
+  </si>
+  <si>
+    <t>Kiểm tra khả năng điều hướng từ màn Home sang module "AI Enhance"</t>
+  </si>
+  <si>
+    <t>1. điều hướng sang module "AI Enhance" bằng 1 trong các cách sau: 
+1.a. chọn image carousel khi hiện banner "AI Enhance"
+1.b. chọn button "AI Enhance" ở fearture compact view 
+1.c. chọn banner "AI Enhance" ở mục "AI Tools"
+1.d. chọn button "AI Enhance" ở mục "Recently Used" (nếu có)</t>
   </si>
   <si>
     <t>- chuyển sang màn "AI Enhance"
@@ -261,7 +261,13 @@
 - hiện modal "Error": check your internet</t>
   </si>
   <si>
-    <t>1.i. chọn button "Collage"</t>
+    <t>F_H_CL</t>
+  </si>
+  <si>
+    <t>Kiểm tra khả năng điều hướng từ màn Home sang module "Collage"</t>
+  </si>
+  <si>
+    <t>1. chọn button "Collage"</t>
   </si>
   <si>
     <t>- sang màn chọn ảnh của module Collage
@@ -269,10 +275,16 @@
 - album default được chọn là "Recent"</t>
   </si>
   <si>
-    <t>sub-ID: F_H_CL</t>
-  </si>
-  <si>
-    <t>1.j.1. chọn button "AI Fill"</t>
+    <t>F_H_AF_NOR</t>
+  </si>
+  <si>
+    <t>Kiểm tra khả năng điều hướng từ màn Home sang module "AI Fill"</t>
+  </si>
+  <si>
+    <t>1. điều hướng sang module "AI Fill" bằng 1 trong số các phương thức sau:
+- chọn button "AI Fill" ở fearture compact view
+- chọn button "AI Fill" ở mục "Recently Used" (nếu có) 
+- chọn banner "AI Fill" tại mục "AI creator"</t>
   </si>
   <si>
     <t>- hiện modal "Try now" của fearture "AI Fill"
@@ -280,20 +292,17 @@
 - layout không bị vỡ/ảnh hưởng khi 'Large text mode' đang được bật</t>
   </si>
   <si>
-    <t>- acount thường</t>
-  </si>
-  <si>
-    <t>2.j.1.a. chọn button "Try now"</t>
+    <t>2.a. chọn button "Try now"</t>
   </si>
   <si>
     <t>- hiện dialog "Chose Image"</t>
   </si>
   <si>
     <t>sub-ID: F_H_AF_NOR_01
-- gồm các step: 1.j.1 -&gt; 2.j.1.a -&gt; 3.j.1.a</t>
-  </si>
-  <si>
-    <t>3.j.1.a. chọn 1 ảnh bất kỳ</t>
+- gồm các step: 1-&gt; 2.a -&gt; 3.a</t>
+  </si>
+  <si>
+    <t>3.a. chọn 1 ảnh bất kỳ</t>
   </si>
   <si>
     <t>- chuyển sang màn "AI Fill"
@@ -302,27 +311,160 @@
 - promt-input text-box trống, chưa có nội dung</t>
   </si>
   <si>
-    <t>2.j.1.b. chọn button "X"</t>
+    <t>2.b. chọn button "X"</t>
   </si>
   <si>
     <t>- ẩn modal "Try now", về màn "Home"</t>
   </si>
   <si>
     <t>sub-ID: F_H_AF_NOR_02
-- gồm các step: 1.j.1 -&gt; 2.j.1.b</t>
-  </si>
-  <si>
-    <t>1.j.2. chọn button "AI Fill"</t>
-  </si>
-  <si>
-    <t>- acount Pro</t>
-  </si>
-  <si>
-    <t>sub-ID:
-F_H_AF_PRO</t>
-  </si>
-  <si>
-    <t>2.j.2 chọn 1 ảnh bất kỳ</t>
+- gồm các step: 1 -&gt; 2.b</t>
+  </si>
+  <si>
+    <t>F_H_AF_PRO</t>
+  </si>
+  <si>
+    <t>1. điều hướng sang module "AI Fill"</t>
+  </si>
+  <si>
+    <t>- account Pro</t>
+  </si>
+  <si>
+    <t>- step 1: truy cập bằng 1 trong số các cách đã nêu ở step 1 tc F_H_AF_NOR</t>
+  </si>
+  <si>
+    <t>F_H_AFT_01</t>
+  </si>
+  <si>
+    <t>Kiểm tra khả năng điều hướng từ màn Home sang module "AI Filter "</t>
+  </si>
+  <si>
+    <t>1. điều hướng sang module AI Fillter bằng 1 trong các cách sau:
+1.a. chọn image carousel khi đang hiện banner "AI Filter" 
+1.b. chọn button "AI Filter" ở fearture compact view 
+1.c. chọn button "AI Filter" ở mục "Recently Used" (nếu có)
+1.d. chọn banner "AI Filter" ở mục "AI creator" 
+1.e. chọn tab "AI Filter" trên tab bar</t>
+  </si>
+  <si>
+    <t>- chuyển sang màn "Choose Style"
+- tab được chọn trên tab bar chuyển sang "AI Filter"
+- Normal (non-pro): các template chỉ dành cho gói pro được đính Badge "Pro"và khóa lại
+- Pro: tất cả các template được mở khóa và không còn Badge "Pro"</t>
+  </si>
+  <si>
+    <t>F_H_AFT_02</t>
+  </si>
+  <si>
+    <t>1. chọn 1 style ở mục "AI Filters"</t>
+  </si>
+  <si>
+    <t>- chuyển sang màn "AI Filter"
+- ảnh input đã được xử lý và gen lại theo style đã chọn</t>
+  </si>
+  <si>
+    <t>F_H_AEX_NOR</t>
+  </si>
+  <si>
+    <t>Kiểm tra khả năng điều hướng từ màn Home sang module "AI Expand"</t>
+  </si>
+  <si>
+    <t>1. điều hướng sang module "AI Expand" bằng 1 trong các cách sau đây: 
+- chọn button "AI Expand"ở fearture compact view
+- chọn button "AI Expand" ở mục "Recently Used" (nếu có)
+- chọn banner "AI Expand" ở mục "AI Tools"</t>
+  </si>
+  <si>
+    <t>- hiện modal "Try now" của fearture "AI Expand"
+- UI modal "Try now" hiển thị đúng theo thiết kế
+- layout không bị vỡ/ảnh hưởng khi 'Large text mode' đang được bật</t>
+  </si>
+  <si>
+    <t>2. chọn button "Try now"</t>
+  </si>
+  <si>
+    <t>- chuyển sang màn "Expand" 
+- ảnh input load thành công, đúng oriantation, không xoay sai chiều</t>
+  </si>
+  <si>
+    <t>F_H_AEX_PRO</t>
+  </si>
+  <si>
+    <t>1. điều hướng sang module "AI Expand"</t>
+  </si>
+  <si>
+    <t>- account pro</t>
+  </si>
+  <si>
+    <t>- step 1: truy cập bằng 1 trong số các cách đã nêu ở step 1 tc F_H_AEX_NOR</t>
+  </si>
+  <si>
+    <t>F_H_AG</t>
+  </si>
+  <si>
+    <t>Kiểm tra khả năng điều hướng từ màn Home sang module "AI Generate"</t>
+  </si>
+  <si>
+    <t>- màn "Home" 
+- đã cấp quyền đầy đủ</t>
+  </si>
+  <si>
+    <t>1. điều hướng sang module "AI Generate" bằng 1 trong các cách sau đây:
+1.a. chọn button "AI Generate" ở fearture compact view
+1.b. chọn tab "AI Generate" ở tab bar 
+1.c. chọn button "AI Generate" ở mục "Recently Used"(nếu có)</t>
+  </si>
+  <si>
+    <t>- chuyển sang màn "Describe"</t>
+  </si>
+  <si>
+    <t>functional test các chức năng còn lại</t>
+  </si>
+  <si>
+    <t>F_H_02</t>
+  </si>
+  <si>
+    <t>kiểm thử chức năng log used-fearture history</t>
+  </si>
+  <si>
+    <t>- màn "Home"</t>
+  </si>
+  <si>
+    <t>1. điều hướng sang 1 fearture bất kỳ</t>
+  </si>
+  <si>
+    <t>- chuyển sang màn hoặc hiển thị các modal ban đầu tương ứng của fearture đó</t>
+  </si>
+  <si>
+    <t>- step1: không cần phải hoàn thành việc điều hướng, chỉ cần chọn button của fearture đó trên màn Home là được</t>
+  </si>
+  <si>
+    <t>2. back về màn "Home"</t>
+  </si>
+  <si>
+    <t>- button của chức nó đó xuất hiện và được đẩy lên thứ tự đầu tiên ở mục "Recently Used"
+- không button chức năng nào bị lặp lại (mỗi fearture chỉ được log 1 lần trong list)</t>
+  </si>
+  <si>
+    <t>F_H_03</t>
+  </si>
+  <si>
+    <t>kiểm thử chức năng link với app "Video Eraser"</t>
+  </si>
+  <si>
+    <t>1. chọn button "Video Object Remover"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- mở "App store" dẫn thẳng đến trang tải app "video eraser" </t>
+  </si>
+  <si>
+    <t>- app "video eraser" chưa được cài đặt</t>
+  </si>
+  <si>
+    <t>- mở app "video eraser"</t>
+  </si>
+  <si>
+    <t>- app "video eraser" đã có trong thiết bị</t>
   </si>
 </sst>
 </file>
@@ -682,7 +824,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -810,6 +952,30 @@
       <left style="medium">
         <color auto="1"/>
       </left>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
       <right style="medium">
         <color auto="1"/>
       </right>
@@ -862,17 +1028,6 @@
         <color auto="1"/>
       </right>
       <top/>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
       <bottom style="medium">
         <color auto="1"/>
       </bottom>
@@ -1015,7 +1170,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1027,34 +1182,34 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="25" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="25" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="26" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1139,13 +1294,19 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1153,150 +1314,294 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" quotePrefix="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" quotePrefix="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1832,504 +2137,838 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="6.3828125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="9.640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="12.375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="29.5546875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="40.1015625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="13.015625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="12.109375" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="9" style="1"/>
+    <col min="1" max="1" width="7.546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="11.5859375" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.375" style="3" customWidth="1"/>
+    <col min="4" max="4" width="29.5546875" style="3" customWidth="1"/>
+    <col min="5" max="5" width="40.1015625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="13.015625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="12.109375" style="3" customWidth="1"/>
+    <col min="8" max="16384" width="9" style="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:7">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="G1" s="50" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" ht="17" spans="1:7">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="40" t="s">
+      <c r="C2" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="41" t="s">
+      <c r="E2" s="79" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="42" t="s">
+      <c r="F2" s="80" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="19"/>
+      <c r="G2" s="51"/>
     </row>
     <row r="3" ht="135" customHeight="1" spans="1:7">
-      <c r="A3" s="7"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="9" t="s">
+      <c r="A3" s="9"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="43" t="s">
+      <c r="E3" s="81" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="20"/>
-      <c r="G3" s="21"/>
+      <c r="F3" s="52"/>
+      <c r="G3" s="53"/>
     </row>
     <row r="4" ht="34" spans="1:7">
-      <c r="A4" s="7"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="9" t="s">
+      <c r="A4" s="9"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="43" t="s">
+      <c r="E4" s="81" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="20"/>
-      <c r="G4" s="21"/>
+      <c r="F4" s="52"/>
+      <c r="G4" s="53"/>
     </row>
     <row r="5" ht="101.75" spans="1:7">
-      <c r="A5" s="10"/>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="12" t="s">
+      <c r="A5" s="12"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="44" t="s">
+      <c r="E5" s="82" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="23"/>
-      <c r="G5" s="24"/>
-    </row>
-    <row r="6" ht="135.75" spans="1:7">
-      <c r="A6" s="13" t="s">
+      <c r="F5" s="49"/>
+      <c r="G5" s="54"/>
+    </row>
+    <row r="6" ht="17.55" spans="1:7">
+      <c r="A6" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="16"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="55"/>
+    </row>
+    <row r="7" ht="103" customHeight="1" spans="1:7">
+      <c r="A7" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="45" t="s">
+      <c r="B7" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="C7" s="83" t="s">
         <v>22</v>
       </c>
-      <c r="E6" s="46" t="s">
+      <c r="D7" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="26"/>
-      <c r="G6" s="27" t="s">
+      <c r="E7" s="84" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="7" ht="185" spans="1:7">
-      <c r="A7" s="13"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="6" t="s">
+      <c r="F7" s="43"/>
+      <c r="G7" s="57"/>
+    </row>
+    <row r="8" ht="185" spans="1:7">
+      <c r="A8" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="47" t="s">
+      <c r="B8" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="F7" s="17"/>
-      <c r="G7" s="29" t="s">
+      <c r="C8" s="78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="8" ht="51.75" spans="1:7">
-      <c r="A8" s="13"/>
-      <c r="B8" s="13"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="12" t="s">
+      <c r="E8" s="85" t="s">
         <v>28</v>
       </c>
-      <c r="E8" s="48" t="s">
+      <c r="F8" s="45"/>
+      <c r="G8" s="51"/>
+    </row>
+    <row r="9" ht="51.75" spans="1:7">
+      <c r="A9" s="22"/>
+      <c r="B9" s="23"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="22"/>
-      <c r="G8" s="31"/>
-    </row>
-    <row r="9" ht="185" spans="1:7">
-      <c r="A9" s="13"/>
-      <c r="B9" s="13"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="6" t="s">
+      <c r="E9" s="86" t="s">
         <v>30</v>
       </c>
-      <c r="E9" s="47" t="s">
-        <v>26</v>
-      </c>
-      <c r="F9" s="17"/>
-      <c r="G9" s="19" t="s">
+      <c r="F9" s="47"/>
+      <c r="G9" s="54"/>
+    </row>
+    <row r="10" ht="202" spans="1:7">
+      <c r="A10" s="6" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="10" ht="101" spans="1:7">
-      <c r="A10" s="13"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="9" t="s">
+      <c r="B10" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="E10" s="49" t="s">
+      <c r="C10" s="78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="F10" s="43" t="s">
+      <c r="E10" s="85" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" s="45"/>
+      <c r="G10" s="87" t="s">
         <v>34</v>
       </c>
-      <c r="G10" s="21"/>
-    </row>
-    <row r="11" ht="34.75" spans="1:7">
-      <c r="A11" s="13"/>
-      <c r="B11" s="13"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="48" t="s">
+    </row>
+    <row r="11" ht="101" spans="1:7">
+      <c r="A11" s="9"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" s="88" t="s">
         <v>35</v>
       </c>
-      <c r="F11" s="44" t="s">
+      <c r="F11" s="81" t="s">
         <v>36</v>
       </c>
-      <c r="G11" s="24"/>
-    </row>
-    <row r="12" ht="34" spans="1:7">
-      <c r="A12" s="13"/>
-      <c r="B12" s="13"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="6" t="s">
+      <c r="G11" s="53"/>
+    </row>
+    <row r="12" ht="34.75" spans="1:7">
+      <c r="A12" s="12"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="86" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="47" t="s">
+      <c r="F12" s="82" t="s">
         <v>38</v>
       </c>
-      <c r="F12" s="17"/>
-      <c r="G12" s="19" t="s">
+      <c r="G12" s="54"/>
+    </row>
+    <row r="13" ht="34" spans="1:7">
+      <c r="A13" s="6" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="13" ht="68" spans="1:7">
-      <c r="A13" s="13"/>
-      <c r="B13" s="13"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="9" t="s">
+      <c r="B13" s="24"/>
+      <c r="C13" s="78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D13" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="E13" s="49" t="s">
+      <c r="E13" s="85" t="s">
         <v>41</v>
       </c>
-      <c r="F13" s="43" t="s">
-        <v>34</v>
-      </c>
-      <c r="G13" s="21"/>
-    </row>
-    <row r="14" ht="34.75" spans="1:7">
-      <c r="A14" s="13"/>
-      <c r="B14" s="13"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="48" t="s">
-        <v>35</v>
-      </c>
-      <c r="F14" s="44" t="s">
+      <c r="F13" s="45"/>
+      <c r="G13" s="87" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" ht="68" spans="1:7">
+      <c r="A14" s="9"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E14" s="88" t="s">
+        <v>43</v>
+      </c>
+      <c r="F14" s="81" t="s">
         <v>36</v>
       </c>
-      <c r="G14" s="24"/>
-    </row>
-    <row r="15" ht="51" spans="1:7">
-      <c r="A15" s="13"/>
-      <c r="B15" s="13"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="6" t="s">
+      <c r="G14" s="53"/>
+    </row>
+    <row r="15" ht="34.75" spans="1:7">
+      <c r="A15" s="12"/>
+      <c r="B15" s="24"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="86" t="s">
+        <v>37</v>
+      </c>
+      <c r="F15" s="82" t="s">
+        <v>38</v>
+      </c>
+      <c r="G15" s="54"/>
+    </row>
+    <row r="16" ht="51" spans="1:7">
+      <c r="A16" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="24"/>
+      <c r="C16" s="78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E16" s="85" t="s">
+        <v>46</v>
+      </c>
+      <c r="F16" s="45"/>
+      <c r="G16" s="87" t="s">
         <v>42</v>
       </c>
-      <c r="E15" s="47" t="s">
-        <v>43</v>
-      </c>
-      <c r="F15" s="17"/>
-      <c r="G15" s="19" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="16" ht="17" spans="1:7">
-      <c r="A16" s="13"/>
-      <c r="B16" s="13"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="E16" s="49" t="s">
-        <v>26</v>
-      </c>
-      <c r="G16" s="21"/>
-    </row>
-    <row r="17" ht="51" spans="1:7">
-      <c r="A17" s="13"/>
-      <c r="B17" s="13"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="E17" s="49" t="s">
+    </row>
+    <row r="17" ht="17" spans="1:7">
+      <c r="A17" s="9"/>
+      <c r="B17" s="24"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="F17" s="43" t="s">
-        <v>34</v>
-      </c>
-      <c r="G17" s="21"/>
-    </row>
-    <row r="18" ht="34.75" spans="1:7">
-      <c r="A18" s="13"/>
-      <c r="B18" s="13"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="48" t="s">
+      <c r="E17" s="88" t="s">
+        <v>28</v>
+      </c>
+      <c r="G17" s="53"/>
+    </row>
+    <row r="18" ht="51" spans="1:7">
+      <c r="A18" s="9"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="F18" s="44" t="s">
+      <c r="E18" s="88" t="s">
+        <v>49</v>
+      </c>
+      <c r="F18" s="81" t="s">
         <v>36</v>
       </c>
-      <c r="G18" s="24"/>
-    </row>
-    <row r="19" ht="168" spans="1:7">
-      <c r="A19" s="13"/>
-      <c r="B19" s="13"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="E19" s="47" t="s">
-        <v>26</v>
-      </c>
-      <c r="F19" s="17"/>
-      <c r="G19" s="19" t="s">
+      <c r="G18" s="53"/>
+    </row>
+    <row r="19" ht="34.75" spans="1:7">
+      <c r="A19" s="12"/>
+      <c r="B19" s="23"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="86" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="20" ht="101.75" spans="1:7">
-      <c r="A20" s="13"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="12" t="s">
+      <c r="F19" s="82" t="s">
+        <v>38</v>
+      </c>
+      <c r="G19" s="54"/>
+    </row>
+    <row r="20" ht="185" spans="1:7">
+      <c r="A20" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E20" s="48" t="s">
+      <c r="B20" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="F20" s="22"/>
-      <c r="G20" s="24"/>
-    </row>
-    <row r="21" ht="101" spans="1:7">
-      <c r="A21" s="13"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="6" t="s">
+      <c r="C20" s="78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="E21" s="47" t="s">
-        <v>26</v>
-      </c>
-      <c r="F21" s="17"/>
-      <c r="G21" s="19" t="s">
+      <c r="E20" s="85" t="s">
+        <v>28</v>
+      </c>
+      <c r="F20" s="45"/>
+      <c r="G20" s="51"/>
+    </row>
+    <row r="21" ht="101.75" spans="1:7">
+      <c r="A21" s="12"/>
+      <c r="B21" s="26"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="E21" s="86" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="22" ht="101.75" spans="1:7">
-      <c r="A22" s="13"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="12" t="s">
+      <c r="F21" s="47"/>
+      <c r="G21" s="54"/>
+    </row>
+    <row r="22" ht="101" spans="1:7">
+      <c r="A22" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="E22" s="48" t="s">
+      <c r="B22" s="26"/>
+      <c r="C22" s="78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D22" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="F22" s="22"/>
-      <c r="G22" s="24"/>
-    </row>
-    <row r="23" ht="185" spans="1:7">
-      <c r="A23" s="13"/>
-      <c r="B23" s="13"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="6" t="s">
+      <c r="E22" s="85" t="s">
+        <v>28</v>
+      </c>
+      <c r="F22" s="45"/>
+      <c r="G22" s="51"/>
+    </row>
+    <row r="23" ht="101.75" spans="1:7">
+      <c r="A23" s="12"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="E23" s="86" t="s">
         <v>57</v>
       </c>
-      <c r="E23" s="47" t="s">
-        <v>26</v>
-      </c>
-      <c r="F23" s="17"/>
-      <c r="G23" s="29" t="s">
+      <c r="F23" s="47"/>
+      <c r="G23" s="54"/>
+    </row>
+    <row r="24" ht="185" spans="1:7">
+      <c r="A24" s="6" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="24" ht="110" customHeight="1" spans="1:7">
-      <c r="A24" s="13"/>
-      <c r="B24" s="13"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="9" t="s">
+      <c r="B24" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="E24" s="49" t="s">
+      <c r="C24" s="78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D24" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="F24" s="43" t="s">
-        <v>34</v>
-      </c>
-      <c r="G24" s="33"/>
-    </row>
-    <row r="25" ht="68.75" spans="1:7">
-      <c r="A25" s="13"/>
-      <c r="B25" s="13"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="48" t="s">
+      <c r="E24" s="85" t="s">
+        <v>28</v>
+      </c>
+      <c r="F24" s="45"/>
+      <c r="G24" s="61"/>
+    </row>
+    <row r="25" ht="110" customHeight="1" spans="1:7">
+      <c r="A25" s="9"/>
+      <c r="B25" s="26"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E25" s="88" t="s">
         <v>61</v>
       </c>
-      <c r="F25" s="44" t="s">
+      <c r="F25" s="81" t="s">
         <v>36</v>
       </c>
-      <c r="G25" s="31"/>
-    </row>
-    <row r="26" ht="68.75" spans="3:7">
-      <c r="C26" s="8"/>
-      <c r="D26" s="15" t="s">
+      <c r="G25" s="62"/>
+    </row>
+    <row r="26" ht="68.75" spans="1:7">
+      <c r="A26" s="12"/>
+      <c r="B26" s="27"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="86" t="s">
         <v>62</v>
       </c>
-      <c r="E26" s="50" t="s">
+      <c r="F26" s="82" t="s">
+        <v>38</v>
+      </c>
+      <c r="G26" s="63"/>
+    </row>
+    <row r="27" ht="101.75" spans="1:7">
+      <c r="A27" s="28" t="s">
         <v>63</v>
       </c>
-      <c r="F26" s="34"/>
-      <c r="G26" s="35" t="s">
+      <c r="B27" s="29" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="27" ht="68" spans="3:7">
-      <c r="C27" s="8"/>
-      <c r="D27" s="6" t="s">
+      <c r="C27" s="89" t="s">
+        <v>22</v>
+      </c>
+      <c r="D27" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="E27" s="41" t="s">
+      <c r="E27" s="90" t="s">
         <v>66</v>
       </c>
-      <c r="F27" s="51" t="s">
+      <c r="F27" s="43"/>
+      <c r="G27" s="57"/>
+    </row>
+    <row r="28" ht="152" spans="1:7">
+      <c r="A28" s="31" t="s">
         <v>67</v>
       </c>
-      <c r="G27" s="19"/>
-    </row>
-    <row r="28" ht="17" spans="3:7">
-      <c r="C28" s="8"/>
-      <c r="D28" s="9" t="s">
+      <c r="B28" s="32" t="s">
         <v>68</v>
       </c>
-      <c r="E28" s="43" t="s">
+      <c r="C28" s="91" t="s">
+        <v>22</v>
+      </c>
+      <c r="D28" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="F28" s="37"/>
-      <c r="G28" s="33" t="s">
+      <c r="E28" s="79" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="29" ht="84" spans="3:7">
-      <c r="C29" s="8"/>
-      <c r="D29" s="9" t="s">
+      <c r="F28" s="92" t="s">
+        <v>12</v>
+      </c>
+      <c r="G28" s="51"/>
+    </row>
+    <row r="29" ht="17" spans="1:7">
+      <c r="A29" s="34"/>
+      <c r="B29" s="35"/>
+      <c r="C29" s="36"/>
+      <c r="D29" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="E29" s="52" t="s">
+      <c r="E29" s="81" t="s">
         <v>72</v>
       </c>
-      <c r="F29" s="37"/>
-      <c r="G29" s="33"/>
-    </row>
-    <row r="30" ht="101.75" spans="3:7">
-      <c r="C30" s="8"/>
-      <c r="D30" s="12" t="s">
+      <c r="F29" s="65"/>
+      <c r="G29" s="62" t="s">
         <v>73</v>
       </c>
-      <c r="E30" s="44" t="s">
+    </row>
+    <row r="30" ht="84" spans="1:7">
+      <c r="A30" s="34"/>
+      <c r="B30" s="35"/>
+      <c r="C30" s="36"/>
+      <c r="D30" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="F30" s="39"/>
-      <c r="G30" s="24" t="s">
+      <c r="E30" s="93" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="31" ht="17" spans="3:7">
-      <c r="C31" s="8"/>
-      <c r="D31" s="6" t="s">
+      <c r="F30" s="65"/>
+      <c r="G30" s="62"/>
+    </row>
+    <row r="31" ht="84.75" spans="1:7">
+      <c r="A31" s="37"/>
+      <c r="B31" s="35"/>
+      <c r="C31" s="38"/>
+      <c r="D31" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="E31" s="41" t="s">
-        <v>26</v>
-      </c>
-      <c r="F31" s="42" t="s">
+      <c r="E31" s="82" t="s">
         <v>77</v>
       </c>
-      <c r="G31" s="19" t="s">
+      <c r="F31" s="67"/>
+      <c r="G31" s="54" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="32" ht="84.75" spans="3:7">
-      <c r="C32" s="8"/>
-      <c r="D32" s="12" t="s">
+    <row r="32" ht="17" spans="1:7">
+      <c r="A32" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="E32" s="44" t="s">
-        <v>72</v>
-      </c>
-      <c r="F32" s="23"/>
-      <c r="G32" s="24"/>
+      <c r="B32" s="35"/>
+      <c r="C32" s="94" t="s">
+        <v>22</v>
+      </c>
+      <c r="D32" s="39" t="s">
+        <v>80</v>
+      </c>
+      <c r="E32" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="F32" s="96" t="s">
+        <v>81</v>
+      </c>
+      <c r="G32" s="97" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="33" ht="84.75" spans="1:7">
+      <c r="A33" s="37"/>
+      <c r="B33" s="40"/>
+      <c r="C33" s="38"/>
+      <c r="D33" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="E33" s="82" t="s">
+        <v>75</v>
+      </c>
+      <c r="F33" s="49"/>
+      <c r="G33" s="54"/>
+    </row>
+    <row r="34" ht="185.75" spans="1:7">
+      <c r="A34" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="B34" s="21" t="s">
+        <v>84</v>
+      </c>
+      <c r="C34" s="98" t="s">
+        <v>22</v>
+      </c>
+      <c r="D34" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="E34" s="90" t="s">
+        <v>86</v>
+      </c>
+      <c r="F34" s="43"/>
+      <c r="G34" s="57"/>
+    </row>
+    <row r="35" ht="17" spans="1:7">
+      <c r="A35" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B35" s="24"/>
+      <c r="C35" s="78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="E35" s="85" t="s">
+        <v>28</v>
+      </c>
+      <c r="F35" s="45"/>
+      <c r="G35" s="51"/>
+    </row>
+    <row r="36" s="1" customFormat="1" ht="51.75" spans="1:7">
+      <c r="A36" s="9"/>
+      <c r="B36" s="24"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="42" t="s">
+        <v>29</v>
+      </c>
+      <c r="E36" s="99" t="s">
+        <v>89</v>
+      </c>
+      <c r="F36" s="72"/>
+      <c r="G36" s="73"/>
+    </row>
+    <row r="37" ht="152" spans="1:7">
+      <c r="A37" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="B37" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="C37" s="78" t="s">
+        <v>22</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="E37" s="79" t="s">
+        <v>93</v>
+      </c>
+      <c r="F37" s="80" t="s">
+        <v>12</v>
+      </c>
+      <c r="G37" s="51"/>
+    </row>
+    <row r="38" ht="28" customHeight="1" spans="1:7">
+      <c r="A38" s="9"/>
+      <c r="B38" s="24"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="E38" s="81" t="s">
+        <v>28</v>
+      </c>
+      <c r="F38" s="52"/>
+      <c r="G38" s="74"/>
+    </row>
+    <row r="39" ht="71" customHeight="1" spans="1:7">
+      <c r="A39" s="12"/>
+      <c r="B39" s="24"/>
+      <c r="C39" s="13"/>
+      <c r="D39" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="E39" s="82" t="s">
+        <v>95</v>
+      </c>
+      <c r="F39" s="49"/>
+      <c r="G39" s="75"/>
+    </row>
+    <row r="40" ht="34" spans="1:7">
+      <c r="A40" s="34" t="s">
+        <v>96</v>
+      </c>
+      <c r="B40" s="24"/>
+      <c r="C40" s="100" t="s">
+        <v>22</v>
+      </c>
+      <c r="D40" s="39" t="s">
+        <v>97</v>
+      </c>
+      <c r="E40" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="F40" s="96" t="s">
+        <v>98</v>
+      </c>
+      <c r="G40" s="101" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="41" ht="83" customHeight="1" spans="1:7">
+      <c r="A41" s="37"/>
+      <c r="B41" s="23"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="E41" s="82" t="s">
+        <v>95</v>
+      </c>
+      <c r="F41" s="49"/>
+      <c r="G41" s="63"/>
+    </row>
+    <row r="42" ht="152.75" spans="1:7">
+      <c r="A42" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="B42" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="C42" s="90" t="s">
+        <v>102</v>
+      </c>
+      <c r="D42" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="E42" s="90" t="s">
+        <v>104</v>
+      </c>
+      <c r="F42" s="43"/>
+      <c r="G42" s="57"/>
+    </row>
+    <row r="43" ht="17.55" spans="1:7">
+      <c r="A43" s="36" t="s">
+        <v>105</v>
+      </c>
+      <c r="B43" s="36"/>
+      <c r="C43" s="36"/>
+      <c r="D43" s="36"/>
+      <c r="E43" s="36"/>
+      <c r="F43" s="36"/>
+      <c r="G43" s="36"/>
+    </row>
+    <row r="44" ht="58" customHeight="1" spans="1:7">
+      <c r="A44" s="31" t="s">
+        <v>106</v>
+      </c>
+      <c r="B44" s="44" t="s">
+        <v>107</v>
+      </c>
+      <c r="C44" s="79" t="s">
+        <v>108</v>
+      </c>
+      <c r="D44" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="E44" s="79" t="s">
+        <v>110</v>
+      </c>
+      <c r="F44" s="76"/>
+      <c r="G44" s="102" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="45" ht="100" customHeight="1" spans="1:7">
+      <c r="A45" s="37"/>
+      <c r="B45" s="46"/>
+      <c r="C45" s="47"/>
+      <c r="D45" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E45" s="82" t="s">
+        <v>113</v>
+      </c>
+      <c r="F45" s="77"/>
+      <c r="G45" s="63"/>
+    </row>
+    <row r="46" ht="51" spans="1:7">
+      <c r="A46" s="31" t="s">
+        <v>114</v>
+      </c>
+      <c r="B46" s="44" t="s">
+        <v>115</v>
+      </c>
+      <c r="C46" s="80" t="s">
+        <v>108</v>
+      </c>
+      <c r="D46" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="E46" s="79" t="s">
+        <v>117</v>
+      </c>
+      <c r="F46" s="79" t="s">
+        <v>118</v>
+      </c>
+      <c r="G46" s="51"/>
+    </row>
+    <row r="47" ht="51.75" spans="1:7">
+      <c r="A47" s="37"/>
+      <c r="B47" s="46"/>
+      <c r="C47" s="49"/>
+      <c r="D47" s="46"/>
+      <c r="E47" s="82" t="s">
+        <v>119</v>
+      </c>
+      <c r="F47" s="82" t="s">
+        <v>120</v>
+      </c>
+      <c r="G47" s="54"/>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="63">
+    <mergeCell ref="A6:G6"/>
+    <mergeCell ref="A43:G43"/>
     <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A6:A25"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="A16:A19"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="A24:A26"/>
+    <mergeCell ref="A28:A31"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A37:A39"/>
+    <mergeCell ref="A40:A41"/>
+    <mergeCell ref="A44:A45"/>
+    <mergeCell ref="A46:A47"/>
     <mergeCell ref="B2:B5"/>
-    <mergeCell ref="B6:B25"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="B10:B19"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="B24:B26"/>
+    <mergeCell ref="B28:B33"/>
+    <mergeCell ref="B34:B36"/>
+    <mergeCell ref="B37:B41"/>
+    <mergeCell ref="B44:B45"/>
+    <mergeCell ref="B46:B47"/>
     <mergeCell ref="C2:C5"/>
-    <mergeCell ref="C6:C32"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="C10:C12"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="C16:C19"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="C24:C26"/>
+    <mergeCell ref="C28:C31"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="C37:C39"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="C44:C45"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="D46:D47"/>
     <mergeCell ref="F2:F5"/>
-    <mergeCell ref="F27:F30"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="G7:G8"/>
-    <mergeCell ref="G9:G11"/>
-    <mergeCell ref="G12:G14"/>
-    <mergeCell ref="G15:G18"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="G21:G22"/>
-    <mergeCell ref="G23:G25"/>
-    <mergeCell ref="G28:G29"/>
-    <mergeCell ref="G31:G32"/>
+    <mergeCell ref="F28:F31"/>
+    <mergeCell ref="F32:F33"/>
+    <mergeCell ref="F37:F39"/>
+    <mergeCell ref="F40:F41"/>
+    <mergeCell ref="F44:F45"/>
+    <mergeCell ref="G10:G12"/>
+    <mergeCell ref="G13:G15"/>
+    <mergeCell ref="G16:G19"/>
+    <mergeCell ref="G20:G21"/>
+    <mergeCell ref="G22:G23"/>
+    <mergeCell ref="G24:G26"/>
+    <mergeCell ref="G29:G30"/>
+    <mergeCell ref="G32:G33"/>
+    <mergeCell ref="G40:G41"/>
+    <mergeCell ref="G44:G45"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>